<commit_message>
feat: implement automation tools for document signing and email distribution in Signar_autofirma and update dashboard template.
</commit_message>
<xml_diff>
--- a/Signar_autofirma/static/plantilla_justificantes.xlsx
+++ b/Signar_autofirma/static/plantilla_justificantes.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,6 +469,11 @@
           <t>fecha de asistencia</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>correo a enviar</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -511,6 +516,11 @@
           <t>25 de maig de 2026</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>destinatario_prueba1@example.com</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -551,6 +561,11 @@
       <c r="H3" t="inlineStr">
         <is>
           <t>26 de maig de 2026</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>destinatario_prueba2@example.com</t>
         </is>
       </c>
     </row>

</xml_diff>